<commit_message>
docs: workplan finalised — shop hardware, paid mentors, own metrology
Adds two tablets as the operator interface and two noise-cancelling
headsets for voice commands on a loud shop floor. Mentorship and
metrology move from Partly to No: the mentors are not free to us and we
own no measuring equipment, so both belong in the funding gap rather
than being counted as covered. Total 5,390 USD.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XuNSKfFGFgyRA5WffAv1uC
</commit_message>
<xml_diff>
--- a/scratch/Forgeron_METI_Workplan.xlsx
+++ b/scratch/Forgeron_METI_Workplan.xlsx
@@ -1295,7 +1295,7 @@
       </c>
       <c r="I29" s="17" t="inlineStr">
         <is>
-          <t>Partly</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J29" s="17" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="I31" s="17" t="inlineStr">
         <is>
-          <t>Partly</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J31" s="17" t="inlineStr">
@@ -1770,24 +1770,24 @@
       </c>
       <c r="C39" s="17" t="inlineStr">
         <is>
-          <t>Software / Digital tools</t>
+          <t>Equipment / Hardware</t>
         </is>
       </c>
       <c r="D39" s="17" t="inlineStr">
         <is>
-          <t>Ollama, FreeCAD, Meshroom (open source)</t>
+          <t>Android tablets (8 GB RAM) as the operator interface, one per pilot shop</t>
         </is>
       </c>
       <c r="E39" s="19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F39" s="17" t="inlineStr">
         <is>
-          <t>months</t>
+          <t>units</t>
         </is>
       </c>
       <c r="G39" s="19" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="H39" s="20">
         <f>IF(OR(E39="",G39=""),"",E39*G39)</f>
@@ -1800,44 +1800,44 @@
       </c>
       <c r="J39" s="17" t="inlineStr">
         <is>
-          <t>Dec 2026</t>
+          <t>Jan 2027</t>
         </is>
       </c>
       <c r="K39" s="17" t="inlineStr">
         <is>
-          <t>Already in use, no licence cost</t>
+          <t>This is how the operator talks to the machine — estimate — to be confirmed by the team</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B40" s="17" t="inlineStr">
         <is>
-          <t>Train the shop operator to run the machine in plain language</t>
+          <t>Run the AI agent fully offline inside the pilot shop</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>Skills / Training</t>
+          <t>Equipment / Hardware</t>
         </is>
       </c>
       <c r="D40" s="17" t="inlineStr">
         <is>
-          <t>Operator training sessions delivered in the shop</t>
+          <t>Headsets with noise-cancelling microphone for voice commands on the shop floor</t>
         </is>
       </c>
       <c r="E40" s="19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F40" s="17" t="inlineStr">
         <is>
-          <t>sessions</t>
+          <t>units</t>
         </is>
       </c>
       <c r="G40" s="19" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="H40" s="20">
         <f>IF(OR(E40="",G40=""),"",E40*G40)</f>
@@ -1855,39 +1855,39 @@
       </c>
       <c r="K40" s="17" t="inlineStr">
         <is>
-          <t>Delivered by our own team</t>
+          <t>A machine shop is loud; voice input needs a directional mic — estimate — to be confirmed by the team</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>Run the AI agent fully offline inside the pilot shop</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>Software / Digital tools</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>Ollama, FreeCAD, Meshroom (open source)</t>
+        </is>
+      </c>
+      <c r="E41" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="B41" s="17" t="inlineStr">
-        <is>
-          <t>Train the shop operator to run the machine in plain language</t>
-        </is>
-      </c>
-      <c r="C41" s="17" t="inlineStr">
-        <is>
-          <t>Technical expertise / Mentorship</t>
-        </is>
-      </c>
-      <c r="D41" s="17" t="inlineStr">
-        <is>
-          <t>Native Bambara speakers to review the closed command lexicon and the safety labels</t>
-        </is>
-      </c>
-      <c r="E41" s="19" t="n">
-        <v>3</v>
-      </c>
       <c r="F41" s="17" t="inlineStr">
         <is>
-          <t>sessions</t>
+          <t>months</t>
         </is>
       </c>
       <c r="G41" s="19" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H41" s="20">
         <f>IF(OR(E41="",G41=""),"",E41*G41)</f>
@@ -1895,49 +1895,49 @@
       </c>
       <c r="I41" s="17" t="inlineStr">
         <is>
-          <t>Partly</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J41" s="17" t="inlineStr">
         <is>
-          <t>Jan 2027</t>
+          <t>Dec 2026</t>
         </is>
       </c>
       <c r="K41" s="17" t="inlineStr">
         <is>
-          <t>Shop operators speak Bambara; emergency-stop and alarm labels must be verified by a native speaker</t>
+          <t>Already in use, no licence cost</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B42" s="17" t="inlineStr">
         <is>
-          <t>Produce at least 5 real customer parts in each shop</t>
+          <t>Train the shop operator to run the machine in plain language</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>Materials / Consumables</t>
+          <t>Skills / Training</t>
         </is>
       </c>
       <c r="D42" s="17" t="inlineStr">
         <is>
-          <t>Aluminium and steel stock for customer parts and trials</t>
+          <t>Operator training sessions delivered in the shop</t>
         </is>
       </c>
       <c r="E42" s="19" t="n">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="F42" s="17" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>sessions</t>
         </is>
       </c>
       <c r="G42" s="19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H42" s="20">
         <f>IF(OR(E42="",G42=""),"",E42*G42)</f>
@@ -1950,44 +1950,44 @@
       </c>
       <c r="J42" s="17" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>Jan 2027</t>
         </is>
       </c>
       <c r="K42" s="17" t="inlineStr">
         <is>
-          <t>Estimate — to be confirmed by the team</t>
+          <t>Delivered by our own team</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B43" s="17" t="inlineStr">
         <is>
-          <t>Produce at least 5 real customer parts in each shop</t>
+          <t>Train the shop operator to run the machine in plain language</t>
         </is>
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
-          <t>Materials / Consumables</t>
+          <t>Technical expertise / Mentorship</t>
         </is>
       </c>
       <c r="D43" s="17" t="inlineStr">
         <is>
-          <t>Carbide cutting tools and replacements</t>
+          <t>Native Bambara speakers to review the closed command lexicon and the safety labels</t>
         </is>
       </c>
       <c r="E43" s="19" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F43" s="17" t="inlineStr">
         <is>
-          <t>tools</t>
+          <t>sessions</t>
         </is>
       </c>
       <c r="G43" s="19" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H43" s="20">
         <f>IF(OR(E43="",G43=""),"",E43*G43)</f>
@@ -2000,12 +2000,12 @@
       </c>
       <c r="J43" s="17" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>Jan 2027</t>
         </is>
       </c>
       <c r="K43" s="17" t="inlineStr">
         <is>
-          <t>Estimate — to be confirmed by the team</t>
+          <t>Shop operators speak Bambara; emergency-stop and alarm labels must be verified by a native speaker</t>
         </is>
       </c>
     </row>
@@ -2020,24 +2020,24 @@
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>Equipment / Hardware</t>
+          <t>Materials / Consumables</t>
         </is>
       </c>
       <c r="D44" s="17" t="inlineStr">
         <is>
-          <t>Metrology set: digital calliper, dial indicator, surface plate</t>
+          <t>Aluminium and steel stock for customer parts and trials</t>
         </is>
       </c>
       <c r="E44" s="19" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="F44" s="17" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="G44" s="19" t="n">
-        <v>250</v>
+        <v>6</v>
       </c>
       <c r="H44" s="20">
         <f>IF(OR(E44="",G44=""),"",E44*G44)</f>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="I44" s="17" t="inlineStr">
         <is>
-          <t>Partly</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J44" s="17" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="K44" s="17" t="inlineStr">
         <is>
-          <t>Needed to prove the parts are within tolerance</t>
+          <t>Estimate — to be confirmed by the team</t>
         </is>
       </c>
     </row>
@@ -2070,24 +2070,24 @@
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>Testing / User access</t>
+          <t>Materials / Consumables</t>
         </is>
       </c>
       <c r="D45" s="17" t="inlineStr">
         <is>
-          <t>Access to the pilot shops and to their real customer orders</t>
+          <t>Carbide cutting tools and replacements</t>
         </is>
       </c>
       <c r="E45" s="19" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="F45" s="17" t="inlineStr">
         <is>
-          <t>months</t>
+          <t>tools</t>
         </is>
       </c>
       <c r="G45" s="19" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H45" s="20">
         <f>IF(OR(E45="",G45=""),"",E45*G45)</f>
@@ -2100,44 +2100,44 @@
       </c>
       <c r="J45" s="17" t="inlineStr">
         <is>
-          <t>Jan 2027</t>
+          <t>Feb 2027</t>
         </is>
       </c>
       <c r="K45" s="17" t="inlineStr">
         <is>
-          <t>This is the core of the pilot</t>
+          <t>Estimate — to be confirmed by the team</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B46" s="17" t="inlineStr">
         <is>
-          <t>Validate the price and build the unit-economics model</t>
+          <t>Produce at least 5 real customer parts in each shop</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>Technical expertise / Mentorship</t>
+          <t>Equipment / Hardware</t>
         </is>
       </c>
       <c r="D46" s="17" t="inlineStr">
         <is>
-          <t>Mentor on pricing and unit economics for hardware ventures</t>
+          <t>Metrology set: digital calliper, dial indicator, surface plate</t>
         </is>
       </c>
       <c r="E46" s="19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F46" s="17" t="inlineStr">
         <is>
-          <t>sessions</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G46" s="19" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="H46" s="20">
         <f>IF(OR(E46="",G46=""),"",E46*G46)</f>
@@ -2145,45 +2145,45 @@
       </c>
       <c r="I46" s="17" t="inlineStr">
         <is>
-          <t>Partly</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J46" s="17" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>Feb 2027</t>
         </is>
       </c>
       <c r="K46" s="17" t="inlineStr">
         <is>
-          <t>Estimate — to be confirmed by the team</t>
+          <t>Needed to prove the parts are within tolerance</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B47" s="17" t="inlineStr">
         <is>
-          <t>Validate the price and build the unit-economics model</t>
+          <t>Produce at least 5 real customer parts in each shop</t>
         </is>
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Testing / User access</t>
         </is>
       </c>
       <c r="D47" s="17" t="inlineStr">
         <is>
-          <t>Costed bill of materials: supplier quotes for mechanical and electronic parts</t>
+          <t>Access to the pilot shops and to their real customer orders</t>
         </is>
       </c>
       <c r="E47" s="19" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F47" s="17" t="inlineStr">
         <is>
-          <t>exercise</t>
+          <t>months</t>
         </is>
       </c>
       <c r="G47" s="19" t="n">
@@ -2200,44 +2200,44 @@
       </c>
       <c r="J47" s="17" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>Jan 2027</t>
         </is>
       </c>
       <c r="K47" s="17" t="inlineStr">
         <is>
-          <t>Our own cost of goods is currently unknown — this is the input the model is missing</t>
+          <t>This is the core of the pilot</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B48" s="17" t="inlineStr">
         <is>
-          <t>Protect the work and pass investor due diligence</t>
+          <t>Validate the price and build the unit-economics model</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>Regulatory / Certification</t>
+          <t>Technical expertise / Mentorship</t>
         </is>
       </c>
       <c r="D48" s="17" t="inlineStr">
         <is>
-          <t>Trademark registration for Forgeron (OAPI)</t>
+          <t>Mentor on pricing and unit economics for hardware ventures</t>
         </is>
       </c>
       <c r="E48" s="19" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F48" s="17" t="inlineStr">
         <is>
-          <t>filing</t>
+          <t>sessions</t>
         </is>
       </c>
       <c r="G48" s="19" t="n">
-        <v>350</v>
+        <v>50</v>
       </c>
       <c r="H48" s="20">
         <f>IF(OR(E48="",G48=""),"",E48*G48)</f>
@@ -2255,27 +2255,27 @@
       </c>
       <c r="K48" s="17" t="inlineStr">
         <is>
-          <t>unknown — fee to be confirmed with OAPI</t>
+          <t>Estimate — to be confirmed by the team</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B49" s="17" t="inlineStr">
         <is>
-          <t>Protect the work and pass investor due diligence</t>
+          <t>Validate the price and build the unit-economics model</t>
         </is>
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>Regulatory / Certification</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D49" s="17" t="inlineStr">
         <is>
-          <t>Machine-safety conformity assessment for commercial sale</t>
+          <t>Costed bill of materials: supplier quotes for mechanical and electronic parts</t>
         </is>
       </c>
       <c r="E49" s="19" t="n">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="F49" s="17" t="inlineStr">
         <is>
-          <t>assessment</t>
+          <t>exercise</t>
         </is>
       </c>
       <c r="G49" s="19" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="H49" s="20">
         <f>IF(OR(E49="",G49=""),"",E49*G49)</f>
@@ -2300,44 +2300,44 @@
       </c>
       <c r="J49" s="17" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="K49" s="17" t="inlineStr">
         <is>
-          <t>unknown — no quote obtained yet</t>
+          <t>Our own cost of goods is currently unknown — this is the input the model is missing</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="17" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B50" s="17" t="inlineStr">
         <is>
-          <t>Document the evidence for the programme and for investors</t>
+          <t>Protect the work and pass investor due diligence</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>Software / Digital tools</t>
+          <t>Regulatory / Certification</t>
         </is>
       </c>
       <c r="D50" s="17" t="inlineStr">
         <is>
-          <t>Mobile data for the team during the pilot</t>
+          <t>Trademark registration for Forgeron (OAPI)</t>
         </is>
       </c>
       <c r="E50" s="19" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F50" s="17" t="inlineStr">
         <is>
-          <t>months</t>
+          <t>filing</t>
         </is>
       </c>
       <c r="G50" s="19" t="n">
-        <v>20</v>
+        <v>350</v>
       </c>
       <c r="H50" s="20">
         <f>IF(OR(E50="",G50=""),"",E50*G50)</f>
@@ -2350,46 +2350,114 @@
       </c>
       <c r="J50" s="17" t="inlineStr">
         <is>
-          <t>Jan 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="K50" s="17" t="inlineStr">
         <is>
-          <t>Estimate — to be confirmed by the team</t>
+          <t>unknown — fee to be confirmed with OAPI</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="17" t="n"/>
-      <c r="B51" s="17" t="n"/>
-      <c r="C51" s="17" t="n"/>
-      <c r="D51" s="17" t="n"/>
-      <c r="E51" s="19" t="n"/>
-      <c r="F51" s="17" t="n"/>
-      <c r="G51" s="19" t="n"/>
+      <c r="A51" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B51" s="17" t="inlineStr">
+        <is>
+          <t>Protect the work and pass investor due diligence</t>
+        </is>
+      </c>
+      <c r="C51" s="17" t="inlineStr">
+        <is>
+          <t>Regulatory / Certification</t>
+        </is>
+      </c>
+      <c r="D51" s="17" t="inlineStr">
+        <is>
+          <t>Machine-safety conformity assessment for commercial sale</t>
+        </is>
+      </c>
+      <c r="E51" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="17" t="inlineStr">
+        <is>
+          <t>assessment</t>
+        </is>
+      </c>
+      <c r="G51" s="19" t="n">
+        <v>500</v>
+      </c>
       <c r="H51" s="20">
         <f>IF(OR(E51="",G51=""),"",E51*G51)</f>
         <v/>
       </c>
-      <c r="I51" s="17" t="n"/>
-      <c r="J51" s="17" t="n"/>
-      <c r="K51" s="17" t="n"/>
+      <c r="I51" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J51" s="17" t="inlineStr">
+        <is>
+          <t>Apr 2027</t>
+        </is>
+      </c>
+      <c r="K51" s="17" t="inlineStr">
+        <is>
+          <t>unknown — no quote obtained yet</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="17" t="n"/>
-      <c r="B52" s="17" t="n"/>
-      <c r="C52" s="17" t="n"/>
-      <c r="D52" s="17" t="n"/>
-      <c r="E52" s="19" t="n"/>
-      <c r="F52" s="17" t="n"/>
-      <c r="G52" s="19" t="n"/>
+      <c r="A52" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>Document the evidence for the programme and for investors</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>Software / Digital tools</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>Mobile data for the team during the pilot</t>
+        </is>
+      </c>
+      <c r="E52" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="F52" s="17" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="G52" s="19" t="n">
+        <v>20</v>
+      </c>
       <c r="H52" s="20">
         <f>IF(OR(E52="",G52=""),"",E52*G52)</f>
         <v/>
       </c>
-      <c r="I52" s="17" t="n"/>
-      <c r="J52" s="17" t="n"/>
-      <c r="K52" s="17" t="n"/>
+      <c r="I52" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J52" s="17" t="inlineStr">
+        <is>
+          <t>Jan 2027</t>
+        </is>
+      </c>
+      <c r="K52" s="17" t="inlineStr">
+        <is>
+          <t>Estimate — to be confirmed by the team</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="17" t="n"/>
@@ -2552,7 +2620,7 @@
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>A laptop with an 8 GB VRAM GPU, so the AI agent runs fully offline inside workshops that have no reliable internet (~USD 1,200).</t>
+          <t>The hardware that lets the AI agent run offline inside a workshop with no reliable internet and no stable power: a laptop with an 8 GB VRAM GPU, two Android tablets as operator interfaces, two noise-cancelling headsets for voice commands on a loud shop floor, and a UPS (~USD 2,190 in total).</t>
         </is>
       </c>
       <c r="C66" s="25" t="n"/>
@@ -2573,7 +2641,7 @@
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>Introductions to machine shops and industrial SMEs in Bamako, plus mentorship on institutional selling. We have a working machine and no customer pipeline — this is our weakest point.</t>
+          <t>Introductions to machine shops and industrial SMEs in Bamako, plus paid mentorship on customer discovery, institutional selling and pricing (~USD 640). We have a working machine and no customer pipeline — this is our weakest point, and the mentors we need are not available to us free of charge.</t>
         </is>
       </c>
       <c r="C67" s="25" t="n"/>
@@ -2594,7 +2662,7 @@
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>Material, cutting tools and metrology to produce and verify the pilot parts (~USD 910), and the safety/certification work needed before we can sell (~USD 850).</t>
+          <t>Material, cutting tools and metrology equipment to produce and verify the pilot parts (~USD 910 — we do not own measuring equipment today), plus the safety and certification work required before we can sell (~USD 850).</t>
         </is>
       </c>
       <c r="C68" s="25" t="n"/>

</xml_diff>